<commit_message>
Update: 2026-09-20 17:08 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -2072,7 +2072,7 @@
         <v>5.12</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>22.9</v>
+        <v>22.8</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4.3</v>
@@ -20185,10 +20185,10 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>6.3</v>
+        <v>5.2</v>
       </c>
       <c r="H77" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J77" t="n">
         <v>3.5</v>
@@ -20200,7 +20200,7 @@
         <v>30</v>
       </c>
       <c r="Q77" t="n">
-        <v>16.7</v>
+        <v>16.6</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update: 2026-10-21 07:01 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -1085,10 +1085,10 @@
         <v>1.047547709</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1.009</v>
+        <v>1.006</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>5.12</v>
+        <v>5.51</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>24.4</v>
@@ -21604,7 +21604,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>default-51d6d6</t>
+          <t>default-CXQrkdu4oQc6aNLKctrnvpf05s3aKZ</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -21614,13 +21614,22 @@
       <c r="H10" t="n">
         <v>80</v>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>1835301600000</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>A German Lager yeast that has it characterized by a clean profile, low ester formation during
+fermentation and medium sulphur production. A good bottom fermenting yeast strain for cold
+fermentation A great choice for all lager styles.</t>
+        </is>
+      </c>
       <c r="K10" t="b">
         <v>0</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -21633,21 +21642,27 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Lallemand (LalBrew)</t>
+          <t>WHC Lab</t>
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="R10" t="n">
+        <v>80</v>
       </c>
       <c r="S10" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="T10" t="n">
+        <v>76</v>
       </c>
       <c r="U10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Diamond Lager</t>
+          <t>Einstein</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -21667,29 +21682,29 @@
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 592000000, "_seconds": 1714216069}</t>
+          <t>{"_nanoseconds": 640000000, "_seconds": 1775809389}</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>EQoOb275xeGHoJJIjjGsUWYLSjWwRD</t>
+          <t>sygWkeOaDxyFuhHuYUsFOB95taxbvR</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 986000000, "_seconds": 1723974355}</t>
+          <t>{"_nanoseconds": 640000000, "_seconds": 1775809389}</t>
         </is>
       </c>
       <c r="AG10" t="n">
-        <v>1723974355986</v>
+        <v>1775809389640</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>2.10.6</t>
+          <t>3.0.0</t>
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>-6</v>
+        <v>2</v>
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
@@ -27638,30 +27653,30 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 538000000, "_seconds": 1697269076}</t>
+          <t>{"_nanoseconds": 320000000, "_seconds": 1787845020}</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>default-90c63c</t>
+          <t>FxymQbqWfYaVaT8ypqgApwGcTjOAXm</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>UuCzoDs2igKSNb78ZPk2m6iGVQT4Eo</t>
+          <t>8ohTm584SLfO1z9IbILXf1d0nQqtl4</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 76000000, "_seconds": 1723974355}</t>
+          <t>{"_nanoseconds": 14000000, "_seconds": 1788116824}</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>1723974355076</v>
+        <v>1788116824014</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2.10.6</t>
+          <t>3.0.1</t>
         </is>
       </c>
       <c r="K49" t="n">
@@ -27672,29 +27687,30 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>-15</v>
+        <v>47.4</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Gelatin</t>
-        </is>
-      </c>
-      <c r="Q49" t="b">
-        <v>1</v>
-      </c>
+          <t>ISY Enhabce</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Fining</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Boil</t>
         </is>
       </c>
       <c r="U49" t="inlineStr"/>

</xml_diff>

<commit_message>
Update: 2026-10-26 07:23 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -14,11 +14,11 @@
     <sheet name="Misc" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$95</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AP$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AP$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2158,8 +2158,68 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>English Porter</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>All Grain</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Ernst Gouws</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>1.047430778</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>1.014</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="L27" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="M27" s="3" t="n">
+        <v>18.58</v>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="P27" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P26"/>
+  <autoFilter ref="A1:P27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2170,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT95"/>
+  <dimension ref="A1:AT101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12433,8 +12493,662 @@
       <c r="AS95" t="inlineStr"/>
       <c r="AT95" t="inlineStr"/>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 499000000, "_seconds": 1706434201}</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>default-e6ba5b8</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>OTZvOBRODuXjmguhpWZUQ4uz2r8zid</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 714000000, "_seconds": 1721546982}</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>1721546982714</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>2.10.6</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M96" t="inlineStr"/>
+      <c r="P96" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>3.2994924</v>
+      </c>
+      <c r="S96" t="n">
+        <v>53</v>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>Base (Maris Otter)</t>
+        </is>
+      </c>
+      <c r="X96" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y96" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z96" t="n">
+        <v>-4.59</v>
+      </c>
+      <c r="AB96" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC96" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>Finest Maris Otter® Ale Malt</t>
+        </is>
+      </c>
+      <c r="AE96" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF96" t="inlineStr">
+        <is>
+          <t>The consistently reliable Maris Otter® continues to provide the qualities expected by the brewer</t>
+        </is>
+      </c>
+      <c r="AG96" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="AH96" t="n">
+        <v>84.18000000000001</v>
+      </c>
+      <c r="AI96" t="n">
+        <v>1.038</v>
+      </c>
+      <c r="AJ96" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="AK96" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL96" t="inlineStr"/>
+      <c r="AM96" t="inlineStr">
+        <is>
+          <t>Crisp</t>
+        </is>
+      </c>
+      <c r="AN96" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO96" t="inlineStr"/>
+      <c r="AP96" t="inlineStr"/>
+      <c r="AQ96" t="inlineStr"/>
+      <c r="AR96" t="inlineStr"/>
+      <c r="AS96" t="inlineStr"/>
+      <c r="AT96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>default-b5ffdd1</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M97" t="inlineStr"/>
+      <c r="P97" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>558.375635</v>
+      </c>
+      <c r="S97" t="n">
+        <v>0</v>
+      </c>
+      <c r="W97" t="inlineStr">
+        <is>
+          <t>Roasted</t>
+        </is>
+      </c>
+      <c r="X97" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB97" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC97" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD97" t="inlineStr">
+        <is>
+          <t>Carafa Special II</t>
+        </is>
+      </c>
+      <c r="AE97" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF97" t="inlineStr">
+        <is>
+          <t>De-husked chocolate malt for a smoother flavor. Adds body, color, aroma. Dark beers, Alts, Bockbiers.</t>
+        </is>
+      </c>
+      <c r="AG97" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="AH97" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="AI97" t="n">
+        <v>1.036</v>
+      </c>
+      <c r="AJ97" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="AK97" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL97" t="inlineStr"/>
+      <c r="AM97" t="inlineStr">
+        <is>
+          <t>Weyermann</t>
+        </is>
+      </c>
+      <c r="AN97" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO97" t="inlineStr"/>
+      <c r="AP97" t="inlineStr"/>
+      <c r="AQ97" t="n">
+        <v>412.8</v>
+      </c>
+      <c r="AR97" t="inlineStr"/>
+      <c r="AS97" t="inlineStr"/>
+      <c r="AT97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 306000000, "_seconds": 1776345994}</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>default-25ba5c7007d</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>1J9fe3tUex3oOKOPk0F51aZTCC6NvP</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 983000000, "_seconds": 1785061179}</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>1785061179983</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="L98" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>61</v>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>Crystal/Caramel</t>
+        </is>
+      </c>
+      <c r="X98" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z98" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="AD98" t="inlineStr">
+        <is>
+          <t>GoldSwaen Classic</t>
+        </is>
+      </c>
+      <c r="AE98" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF98" t="inlineStr">
+        <is>
+          <t>5-10% for dark beers, 1-5% for light beer, Pale Ale 20%</t>
+        </is>
+      </c>
+      <c r="AG98" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH98" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="AI98" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AJ98" t="n">
+        <v>73.9130435</v>
+      </c>
+      <c r="AL98" t="inlineStr"/>
+      <c r="AM98" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
+      <c r="AN98" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO98" t="inlineStr"/>
+      <c r="AP98" t="inlineStr"/>
+      <c r="AQ98" t="inlineStr"/>
+      <c r="AR98" t="inlineStr"/>
+      <c r="AS98" t="inlineStr"/>
+      <c r="AT98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>default-d2c0778</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="L99" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr"/>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>Oats, Flaked</t>
+        </is>
+      </c>
+      <c r="AE99" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF99" t="inlineStr"/>
+      <c r="AG99" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AH99" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="AI99" t="n">
+        <v>1.0391</v>
+      </c>
+      <c r="AJ99" t="n">
+        <v>85</v>
+      </c>
+      <c r="AL99" t="inlineStr"/>
+      <c r="AM99" t="inlineStr">
+        <is>
+          <t>Briess</t>
+        </is>
+      </c>
+      <c r="AN99" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO99" t="inlineStr"/>
+      <c r="AP99" t="inlineStr"/>
+      <c r="AQ99" t="inlineStr"/>
+      <c r="AR99" t="inlineStr"/>
+      <c r="AS99" t="inlineStr"/>
+      <c r="AT99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 212000000, "_seconds": 1775499019}</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>default-c5e48c4</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>9mGQgdZMjKAOZQSjsXo7x5DVWTbPaC</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 714000000, "_seconds": 1777108185}</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>1777108185714</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>3.0.0</t>
+        </is>
+      </c>
+      <c r="K100" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="M100" t="inlineStr"/>
+      <c r="P100" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>529.4416244</v>
+      </c>
+      <c r="S100" t="n">
+        <v>0</v>
+      </c>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t>Roasted</t>
+        </is>
+      </c>
+      <c r="X100" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y100" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z100" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AB100" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC100" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD100" t="inlineStr">
+        <is>
+          <t>Chocolate Malt</t>
+        </is>
+      </c>
+      <c r="AE100" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF100" t="inlineStr">
+        <is>
+          <t>Gives dry, toasty flavours to rich, dark beers</t>
+        </is>
+      </c>
+      <c r="AG100" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="AH100" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="AI100" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="AJ100" t="n">
+        <v>72</v>
+      </c>
+      <c r="AK100" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL100" t="inlineStr"/>
+      <c r="AM100" t="inlineStr">
+        <is>
+          <t>Crisp</t>
+        </is>
+      </c>
+      <c r="AN100" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO100" t="inlineStr"/>
+      <c r="AP100" t="inlineStr"/>
+      <c r="AQ100" t="inlineStr"/>
+      <c r="AR100" t="inlineStr"/>
+      <c r="AS100" t="inlineStr"/>
+      <c r="AT100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 593000000, "_seconds": 1776345977}</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>default-29dda1b5335</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>R3yyMXfk1baparTfJ2ej9HajPEgito</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 919000000, "_seconds": 1781339588}</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>1781339588919</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="L101" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>329.949239</v>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>Crystal/Caramel</t>
+        </is>
+      </c>
+      <c r="X101" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z101" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AD101" t="inlineStr">
+        <is>
+          <t>BlackSwaen Coffee</t>
+        </is>
+      </c>
+      <c r="AE101" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF101" t="inlineStr"/>
+      <c r="AG101" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH101" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="AI101" t="n">
+        <v>1.028</v>
+      </c>
+      <c r="AJ101" t="n">
+        <v>60.8695652</v>
+      </c>
+      <c r="AL101" t="inlineStr"/>
+      <c r="AM101" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
+      <c r="AN101" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO101" t="inlineStr"/>
+      <c r="AP101" t="inlineStr"/>
+      <c r="AQ101" t="n">
+        <v>244.1</v>
+      </c>
+      <c r="AR101" t="inlineStr"/>
+      <c r="AS101" t="inlineStr"/>
+      <c r="AT101" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AT95"/>
+  <autoFilter ref="A1:AT101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12445,7 +13159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP80"/>
+  <dimension ref="A1:AP82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -20566,8 +21280,226 @@
       <c r="AO80" t="inlineStr"/>
       <c r="AP80" t="inlineStr"/>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>default-J80zzFn0TQEAwwaQuzMQsRYzrIvBOC</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H81" t="n">
+        <v>15</v>
+      </c>
+      <c r="J81" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N81" t="b">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Hallertau Perle</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>A dual-purpose hop that offers great bittering properties as well as a well-rounded aroma profile. Aroma: Herbal - tea, pepper, floral, citrus, earthy, woody, grassy, caramel Alpha Acid: 4.0 - 9.0% Beta Acid: 2.5 - 4.5% Total Oil: 0.5 - 1.3 ml/100g</t>
+        </is>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr"/>
+      <c r="Z81" t="n">
+        <v>60</v>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB81" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC81" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD81" t="inlineStr"/>
+      <c r="AE81" t="inlineStr"/>
+      <c r="AF81" t="n">
+        <v>2024</v>
+      </c>
+      <c r="AG81" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 223000000, "_seconds": 1778682625}</t>
+        </is>
+      </c>
+      <c r="AH81" t="inlineStr">
+        <is>
+          <t>G1hAXrUVQhnMlGnAla7zTuBYG3dJVx</t>
+        </is>
+      </c>
+      <c r="AI81" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 715000000, "_seconds": 1789895043}</t>
+        </is>
+      </c>
+      <c r="AJ81" t="n">
+        <v>1789895043715</v>
+      </c>
+      <c r="AK81" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="AL81" t="n">
+        <v>138</v>
+      </c>
+      <c r="AM81" t="inlineStr"/>
+      <c r="AN81" t="inlineStr"/>
+      <c r="AO81" t="inlineStr"/>
+      <c r="AP81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>default-J80zzFn0TQEAwwaQuzMQsRYzrIvBOC</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H82" t="n">
+        <v>15</v>
+      </c>
+      <c r="J82" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N82" t="b">
+        <v>0</v>
+      </c>
+      <c r="O82" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Hallertau Perle</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>A dual-purpose hop that offers great bittering properties as well as a well-rounded aroma profile. Aroma: Herbal - tea, pepper, floral, citrus, earthy, woody, grassy, caramel Alpha Acid: 4.0 - 9.0% Beta Acid: 2.5 - 4.5% Total Oil: 0.5 - 1.3 ml/100g</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="X82" t="inlineStr"/>
+      <c r="Z82" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB82" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC82" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD82" t="inlineStr"/>
+      <c r="AE82" t="inlineStr"/>
+      <c r="AF82" t="n">
+        <v>2024</v>
+      </c>
+      <c r="AG82" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 223000000, "_seconds": 1778682625}</t>
+        </is>
+      </c>
+      <c r="AH82" t="inlineStr">
+        <is>
+          <t>G1hAXrUVQhnMlGnAla7zTuBYG3dJVx</t>
+        </is>
+      </c>
+      <c r="AI82" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 715000000, "_seconds": 1789895043}</t>
+        </is>
+      </c>
+      <c r="AJ82" t="n">
+        <v>1789895043715</v>
+      </c>
+      <c r="AK82" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="AL82" t="n">
+        <v>138</v>
+      </c>
+      <c r="AM82" t="inlineStr"/>
+      <c r="AN82" t="inlineStr"/>
+      <c r="AO82" t="inlineStr"/>
+      <c r="AP82" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AP80"/>
+  <autoFilter ref="A1:AP82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20578,7 +21510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL26"/>
+  <dimension ref="A1:AL27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -23569,8 +24501,115 @@
       <c r="AK26" t="inlineStr"/>
       <c r="AL26" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Yeast</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>default-clIP1PsQiKPjtT5G8QaCqk0OjM2WlR</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="n">
+        <v>70</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Clean, aggressive, attenuative, ABV tolerant and highly flocculant. This yeast is the go-to house yeast for many microbreweries. This English style yeast provides the backbone for everything from IPA's to stouts to barleywines. Equivalent: Imperial House, White Labs WLP007 Dry English Ale, Wyeast 1098 British, Omega British Ale I</t>
+        </is>
+      </c>
+      <c r="K27" t="b">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Dry</t>
+        </is>
+      </c>
+      <c r="N27" t="b">
+        <v>0</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>WHC Lab</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>12</v>
+      </c>
+      <c r="R27" t="n">
+        <v>80</v>
+      </c>
+      <c r="S27" t="n">
+        <v>21</v>
+      </c>
+      <c r="T27" t="n">
+        <v>73</v>
+      </c>
+      <c r="U27" t="n">
+        <v>16</v>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>British Pub Ale</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>Ale</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>pkg</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
+      <c r="AJ27" t="n">
+        <v>13</v>
+      </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>Stout, IPA, Pale Ale, Brown Ale, Red Ale, Imperial Stout</t>
+        </is>
+      </c>
+      <c r="AL27" t="n">
+        <v>250</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AL26"/>
+  <autoFilter ref="A1:AL27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23581,7 +24620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB146"/>
+  <dimension ref="A1:AB152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -35831,8 +36870,529 @@
       <c r="AA146" t="inlineStr"/>
       <c r="AB146" t="inlineStr"/>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 20000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>default-2302b0</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>dHzf3qHIzqCVtmbVlXqvCaYqHnAPxv</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 69000000, "_seconds": 1781339599}</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>1781339599069</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K147" t="n">
+        <v>2</v>
+      </c>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="b">
+        <v>0</v>
+      </c>
+      <c r="N147" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>Baking Soda (NaHCO3)</t>
+        </is>
+      </c>
+      <c r="Q147" t="b">
+        <v>0</v>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U147" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y147" t="inlineStr"/>
+      <c r="Z147" t="inlineStr"/>
+      <c r="AA147" t="inlineStr"/>
+      <c r="AB147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>default-3b1827</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>xD9x1qmhYt1snySGFEG5hYH8K6gljD</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 647000000, "_seconds": 1789895044}</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>1789895044647</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="K148" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M148" t="b">
+        <v>0</v>
+      </c>
+      <c r="N148" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Calcium Chloride (CaCl2)</t>
+        </is>
+      </c>
+      <c r="Q148" t="b">
+        <v>0</v>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U148" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y148" t="inlineStr"/>
+      <c r="Z148" t="inlineStr"/>
+      <c r="AA148" t="inlineStr"/>
+      <c r="AB148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>default-1f88df</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>gPQRHI0XC908S70pJd3aPLDlxNrL00</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 309000000, "_seconds": 1789895044}</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>1789895044309</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="K149" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L149" t="inlineStr"/>
+      <c r="M149" t="b">
+        <v>0</v>
+      </c>
+      <c r="N149" t="n">
+        <v>929.5</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>Gypsum (CaSO4)</t>
+        </is>
+      </c>
+      <c r="Q149" t="b">
+        <v>0</v>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U149" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y149" t="inlineStr"/>
+      <c r="Z149" t="inlineStr"/>
+      <c r="AA149" t="inlineStr"/>
+      <c r="AB149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>default-07adb1</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>1f3RTpuz73jj4GfdSrqo9SZDV92mBR</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 34000000, "_seconds": 1789895045}</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>1789895045034</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="K150" t="n">
+        <v>2</v>
+      </c>
+      <c r="L150" t="n">
+        <v>80</v>
+      </c>
+      <c r="M150" t="b">
+        <v>0</v>
+      </c>
+      <c r="N150" t="n">
+        <v>334</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Lactic Acid</t>
+        </is>
+      </c>
+      <c r="Q150" t="b">
+        <v>0</v>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U150" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y150" t="inlineStr"/>
+      <c r="Z150" t="inlineStr"/>
+      <c r="AA150" t="inlineStr"/>
+      <c r="AB150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>default-5adf6e</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>XqJmJZ27RihaOgdZypjjCAeZ5Ybero</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 404000000, "_seconds": 1789895045}</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>1789895045404</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="K151" t="n">
+        <v>1</v>
+      </c>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="b">
+        <v>0</v>
+      </c>
+      <c r="N151" t="n">
+        <v>4</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Irish Moss</t>
+        </is>
+      </c>
+      <c r="P151" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q151" t="b">
+        <v>0</v>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>Fining</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr"/>
+      <c r="Y151" t="inlineStr"/>
+      <c r="Z151" t="inlineStr"/>
+      <c r="AA151" t="inlineStr"/>
+      <c r="AB151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>xlBmZbXhzbuHWfN1GoclwNdsgM9yT6</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summer stout </t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 67000000, "_seconds": 1775809134}</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>default-yn-wln1000</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>kdl08EEBMhKVgFHBmTNKK0S3PJxlNw</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 532000000, "_seconds": 1789895046}</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>1789895046532</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="K152" t="n">
+        <v>5</v>
+      </c>
+      <c r="L152" t="inlineStr"/>
+      <c r="M152" t="b">
+        <v>0</v>
+      </c>
+      <c r="N152" t="n">
+        <v>77.23999999999999</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Yeast Nutrient (WLN1000)</t>
+        </is>
+      </c>
+      <c r="P152" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q152" t="b">
+        <v>0</v>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U152" t="inlineStr"/>
+      <c r="V152" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Y152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">White Labs Yeast Nutrient is used to increase the health of yeast, this improves fermentation and re-pitching performance. It contains diammonium phosphate (DAP), essential vitamins and co-factors, nitrogen, amino acids, proteins, peptides, and minerals. An effective boost for first and/or late-generation yeast slurry. If the grist is not 100% malt, then White Labs Yeast Nutrient can help make up for the lack of nutrients.
+We recommend using traditional finings agents for most fermentations. If you are still struggling with unwanted haze, filtration may be necessary. </t>
+        </is>
+      </c>
+      <c r="Z152" t="inlineStr"/>
+      <c r="AA152" t="inlineStr"/>
+      <c r="AB152" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB146"/>
+  <autoFilter ref="A1:AB152"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: 2026-10-29 07:59 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -28545,30 +28545,30 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>tRIJHPH0GJDvX68lIylAwbxCHqdx60</t>
+          <t>xD9x1qmhYt1snySGFEG5hYH8K6gljD</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 930000000, "_seconds": 1704369575}</t>
+          <t>{"_nanoseconds": 647000000, "_seconds": 1789895044}</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>1704369575930</v>
+        <v>1789895044647</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2.10.4</t>
+          <t>3.1.0</t>
         </is>
       </c>
       <c r="K46" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="M46" t="b">
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>32.5</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -28596,9 +28596,6 @@
       <c r="U46" t="b">
         <v>1</v>
       </c>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
-      <c r="X46" t="inlineStr"/>
       <c r="Y46" t="inlineStr"/>
       <c r="Z46" t="inlineStr"/>
       <c r="AA46" t="inlineStr"/>
@@ -28632,20 +28629,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>lcvTqdMfO6NPRj6JBJoHMhZuaJN2Fj</t>
+          <t>gPQRHI0XC908S70pJd3aPLDlxNrL00</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 428000000, "_seconds": 1772634485}</t>
+          <t>{"_nanoseconds": 309000000, "_seconds": 1789895044}</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>1772634485428</v>
+        <v>1789895044309</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2.20.2</t>
+          <t>3.1.0</t>
         </is>
       </c>
       <c r="K47" t="n">
@@ -28656,7 +28653,7 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>929.5</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -28717,24 +28714,24 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>eIuDGEasVf2TMzwhyNhxT2RGDDKeIc</t>
+          <t>1f3RTpuz73jj4GfdSrqo9SZDV92mBR</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 497000000, "_seconds": 1772634487}</t>
+          <t>{"_nanoseconds": 34000000, "_seconds": 1789895045}</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>1772634487497</v>
+        <v>1789895045034</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2.20.2</t>
+          <t>3.1.0</t>
         </is>
       </c>
       <c r="K48" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="L48" t="n">
         <v>80</v>
@@ -28743,7 +28740,7 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>334</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>

</xml_diff>